<commit_message>
feat: error in ExcelRepository change serch for contain
</commit_message>
<xml_diff>
--- a/cosatcal/CosatCal_dati.xlsx
+++ b/cosatcal/CosatCal_dati.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="4"/>
+    <workbookView activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="LEGGIMI" sheetId="1" r:id="rId1"/>
@@ -2430,7 +2430,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B298"/>
+  <dimension ref="A1:B297"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.00390625" customWidth="1"/>
@@ -3649,13 +3649,9 @@
       <c r="A297" s="4"/>
       <c r="B297" s="4"/>
     </row>
-    <row r="298">
-      <c r="A298" s="4"/>
-      <c r="B298" s="4"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valore non valido" error="Inserire un prezzo &gt;= 0 (€/kg)." sqref="B2:B298">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valore non valido" error="Inserire un prezzo &gt;= 0 (€/kg)." sqref="B2:B297">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Applied final corrections to improve the way informations is returned and displayed
</commit_message>
<xml_diff>
--- a/cosatcal/CosatCal_dati.xlsx
+++ b/cosatcal/CosatCal_dati.xlsx
@@ -2430,7 +2430,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B297"/>
+  <dimension ref="A1:B290"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.00390625" customWidth="1"/>
@@ -3621,37 +3621,9 @@
       <c r="A290" s="4"/>
       <c r="B290" s="4"/>
     </row>
-    <row r="291">
-      <c r="A291" s="4"/>
-      <c r="B291" s="4"/>
-    </row>
-    <row r="292">
-      <c r="A292" s="4"/>
-      <c r="B292" s="4"/>
-    </row>
-    <row r="293">
-      <c r="A293" s="4"/>
-      <c r="B293" s="4"/>
-    </row>
-    <row r="294">
-      <c r="A294" s="4"/>
-      <c r="B294" s="4"/>
-    </row>
-    <row r="295">
-      <c r="A295" s="4"/>
-      <c r="B295" s="4"/>
-    </row>
-    <row r="296">
-      <c r="A296" s="4"/>
-      <c r="B296" s="4"/>
-    </row>
-    <row r="297">
-      <c r="A297" s="4"/>
-      <c r="B297" s="4"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valore non valido" error="Inserire un prezzo &gt;= 0 (€/kg)." sqref="B2:B297">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valore non valido" error="Inserire un prezzo &gt;= 0 (€/kg)." sqref="B2:B6 B7:B290">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>